<commit_message>
Tables, séquence 1 : commentaire utile après une bonne explication (pourquoi ça marche, autre façon, méthode préférée)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E92HNC9FUW2VcTzfmpL2ox
</commit_message>
<xml_diff>
--- a/data/table-8-questions.xlsx
+++ b/data/table-8-questions.xlsx
@@ -106,7 +106,7 @@
     <t xml:space="preserve">• Stratégie : facultatif, pour les choix justes. Le code (onglet « Stratégies ») sert à écrire la phrase de la fiche mémo.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Explication si choisi : affichée quand l’élève choisit un choix faux.</t>
+    <t xml:space="preserve">• Explication si choisi : pour un choix faux, ce qui ne va pas ; pour un choix juste, pourquoi la méthode marche. Vide pour un choix juste : la plateforme écrit un commentaire automatique selon la stratégie.</t>
   </si>
   <si>
     <t xml:space="preserve">Repères dans les textes (l’élève choisit au début d’écrire 8 × 3 ou 3 × 8)</t>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>

</xml_diff>

<commit_message>
Tables, séquence 1 : « Autre façon » jamais identique au choix ni au commentaire ; un choix faux dans chaque question par défaut
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E92HNC9FUW2VcTzfmpL2ox
</commit_message>
<xml_diff>
--- a/data/table-8-questions.xlsx
+++ b/data/table-8-questions.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Stratégies" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Tables!$A$1:$J$41</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Tables!$A$1:$J$48</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="118">
   <si>
     <t xml:space="preserve">Questions de la séquence 1 d’Explorer — table de 8</t>
   </si>
@@ -289,6 +289,12 @@
     <t xml:space="preserve">40 − 8 = 32 : j’enlève 8 au résultat suivant.</t>
   </si>
   <si>
+    <t xml:space="preserve">24 + 4 = 32.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non : 24 + 4 = 28. Dans la table de 8, on ajoute 8, pas 4 : 24 + 8 = 32.</t>
+  </si>
+  <si>
     <t xml:space="preserve">80 + 8 = 88 : 10 fois 8, plus encore 8.</t>
   </si>
   <si>
@@ -298,6 +304,12 @@
     <t xml:space="preserve">{autre} = 88.</t>
   </si>
   <si>
+    <t xml:space="preserve">80 + 11 = 88.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non : 80 + 11 = 91. On part de 80 et on ajoute 8 : 80 + 8 = 88.</t>
+  </si>
+  <si>
     <t xml:space="preserve">56 + 8 = 64 : j’ajoute 8 au résultat précédent.</t>
   </si>
   <si>
@@ -307,6 +319,12 @@
     <t xml:space="preserve">72 − 8 = 64 : j’enlève 8 au résultat suivant.</t>
   </si>
   <si>
+    <t xml:space="preserve">8 + 8 = 64.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non : 8 + 8 = 16, c’est {×2}. Pour 64, il faut prendre 8 fois 8.</t>
+  </si>
+  <si>
     <t xml:space="preserve">40 + 8 = 48 : j’ajoute 8 au résultat précédent.</t>
   </si>
   <si>
@@ -316,6 +334,12 @@
     <t xml:space="preserve">56 − 8 = 48 : j’enlève 8 au résultat suivant.</t>
   </si>
   <si>
+    <t xml:space="preserve">40 + 6 = 48.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non : 40 + 6 = 46. Dans la table de 8, on ajoute 8, pas 6 : 40 + 8 = 48.</t>
+  </si>
+  <si>
     <t xml:space="preserve">48 + 8 = 56 : j’ajoute 8 au résultat précédent.</t>
   </si>
   <si>
@@ -325,6 +349,12 @@
     <t xml:space="preserve">64 − 8 = 56 : j’enlève 8 au résultat suivant.</t>
   </si>
   <si>
+    <t xml:space="preserve">48 + 7 = 56.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non : 48 + 7 = 55. Dans la table de 8, on ajoute 8, pas 7 : 48 + 8 = 56.</t>
+  </si>
+  <si>
     <t xml:space="preserve">64 + 8 = 72 : j’ajoute 8 au résultat précédent.</t>
   </si>
   <si>
@@ -334,6 +364,12 @@
     <t xml:space="preserve">80 − 8 = 72 : j’enlève 8 au résultat suivant.</t>
   </si>
   <si>
+    <t xml:space="preserve">64 + 9 = 72.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non : 64 + 9 = 73. Dans la table de 8, on ajoute 8, pas 9 : 64 + 8 = 72.</t>
+  </si>
+  <si>
     <t xml:space="preserve">88 + 8 = 96 : j’ajoute 8 au résultat précédent.</t>
   </si>
   <si>
@@ -344,6 +380,12 @@
   </si>
   <si>
     <t xml:space="preserve">pose</t>
+  </si>
+  <si>
+    <t xml:space="preserve">80 + 12 = 96.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non : 80 + 12 = 92. On découpe 12 en 10 + 2 : 80 + 16 = 96.</t>
   </si>
   <si>
     <t xml:space="preserve">Code</t>
@@ -1058,7 +1100,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -1809,37 +1851,37 @@
       </c>
       <c r="J23" s="5"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B24" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="C24" s="9" t="n">
-        <v>11</v>
-      </c>
-      <c r="D24" s="10" t="str">
+    <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" s="6" t="str">
         <f aca="false">"8 × "&amp;C24</f>
-        <v>8 × 11</v>
-      </c>
-      <c r="E24" s="10" t="n">
+        <v>8 × 4</v>
+      </c>
+      <c r="E24" s="6" t="n">
         <f aca="false">VALUE(MID(A24,7,2))*C24</f>
-        <v>88</v>
-      </c>
-      <c r="F24" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G24" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="H24" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I24" s="9" t="s">
+      <c r="H24" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="J24" s="9"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
@@ -1860,7 +1902,7 @@
         <v>88</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G25" s="9" t="s">
         <v>74</v>
@@ -1869,7 +1911,7 @@
         <v>38</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>54</v>
+        <v>75</v>
       </c>
       <c r="J25" s="9"/>
     </row>
@@ -1892,82 +1934,82 @@
         <v>88</v>
       </c>
       <c r="F26" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G26" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="H26" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I26" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="J26" s="9"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C27" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="D27" s="10" t="str">
+        <f aca="false">"8 × "&amp;C27</f>
+        <v>8 × 11</v>
+      </c>
+      <c r="E27" s="10" t="n">
+        <f aca="false">VALUE(MID(A27,7,2))*C27</f>
+        <v>88</v>
+      </c>
+      <c r="F27" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G26" s="9" t="s">
+      <c r="G27" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H26" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I26" s="9" t="s">
+      <c r="H27" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I27" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="J26" s="9"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B27" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="C27" s="5" t="n">
+      <c r="J27" s="9"/>
+    </row>
+    <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D27" s="6" t="str">
-        <f aca="false">"8 × "&amp;C27</f>
-        <v>8 × 8</v>
-      </c>
-      <c r="E27" s="6" t="n">
-        <f aca="false">VALUE(MID(A27,7,2))*C27</f>
-        <v>64</v>
-      </c>
-      <c r="F27" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="H27" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="I27" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="J27" s="5"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B28" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="C28" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="D28" s="6" t="str">
+      <c r="C28" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="D28" s="10" t="str">
         <f aca="false">"8 × "&amp;C28</f>
-        <v>8 × 8</v>
-      </c>
-      <c r="E28" s="6" t="n">
+        <v>8 × 11</v>
+      </c>
+      <c r="E28" s="10" t="n">
         <f aca="false">VALUE(MID(A28,7,2))*C28</f>
-        <v>64</v>
-      </c>
-      <c r="F28" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="H28" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="I28" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J28" s="5"/>
+        <v>88</v>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G28" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="H28" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="I28" s="9"/>
+      <c r="J28" s="9" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
@@ -1988,405 +2030,629 @@
         <v>64</v>
       </c>
       <c r="F29" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="H29" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="J29" s="5"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D30" s="6" t="str">
+        <f aca="false">"8 × "&amp;C30</f>
+        <v>8 × 8</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <f aca="false">VALUE(MID(A30,7,2))*C30</f>
+        <v>64</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="H30" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J30" s="5"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D31" s="6" t="str">
+        <f aca="false">"8 × "&amp;C31</f>
+        <v>8 × 8</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <f aca="false">VALUE(MID(A31,7,2))*C31</f>
+        <v>64</v>
+      </c>
+      <c r="F31" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G29" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="H29" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="I29" s="5" t="s">
+      <c r="G31" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="H31" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I31" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="J29" s="5"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B30" s="9" t="n">
+      <c r="J31" s="5"/>
+    </row>
+    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D32" s="6" t="str">
+        <f aca="false">"8 × "&amp;C32</f>
+        <v>8 × 8</v>
+      </c>
+      <c r="E32" s="6" t="n">
+        <f aca="false">VALUE(MID(A32,7,2))*C32</f>
+        <v>64</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="I32" s="5"/>
+      <c r="J32" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="C30" s="9" t="n">
+      <c r="C33" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="D30" s="10" t="str">
-        <f aca="false">"8 × "&amp;C30</f>
+      <c r="D33" s="10" t="str">
+        <f aca="false">"8 × "&amp;C33</f>
         <v>8 × 6</v>
       </c>
-      <c r="E30" s="10" t="n">
-        <f aca="false">VALUE(MID(A30,7,2))*C30</f>
+      <c r="E33" s="10" t="n">
+        <f aca="false">VALUE(MID(A33,7,2))*C33</f>
         <v>48</v>
       </c>
-      <c r="F30" s="9" t="n">
+      <c r="F33" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G30" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="H30" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I30" s="9" t="s">
+      <c r="G33" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="H33" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I33" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="J30" s="9"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B31" s="9" t="n">
+      <c r="J33" s="9"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="C31" s="9" t="n">
+      <c r="C34" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="D31" s="10" t="str">
-        <f aca="false">"8 × "&amp;C31</f>
+      <c r="D34" s="10" t="str">
+        <f aca="false">"8 × "&amp;C34</f>
         <v>8 × 6</v>
       </c>
-      <c r="E31" s="10" t="n">
-        <f aca="false">VALUE(MID(A31,7,2))*C31</f>
+      <c r="E34" s="10" t="n">
+        <f aca="false">VALUE(MID(A34,7,2))*C34</f>
         <v>48</v>
       </c>
-      <c r="F31" s="9" t="n">
+      <c r="F34" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="G31" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="H31" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I31" s="9" t="s">
+      <c r="G34" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="H34" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I34" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="J31" s="9"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B32" s="9" t="n">
+      <c r="J34" s="9"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B35" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="C32" s="9" t="n">
+      <c r="C35" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="D32" s="10" t="str">
-        <f aca="false">"8 × "&amp;C32</f>
+      <c r="D35" s="10" t="str">
+        <f aca="false">"8 × "&amp;C35</f>
         <v>8 × 6</v>
       </c>
-      <c r="E32" s="10" t="n">
-        <f aca="false">VALUE(MID(A32,7,2))*C32</f>
+      <c r="E35" s="10" t="n">
+        <f aca="false">VALUE(MID(A35,7,2))*C35</f>
         <v>48</v>
       </c>
-      <c r="F32" s="9" t="n">
+      <c r="F35" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G32" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="H32" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I32" s="9" t="s">
+      <c r="G35" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="H35" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I35" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="J32" s="9"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B33" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="C33" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="D33" s="6" t="str">
-        <f aca="false">"8 × "&amp;C33</f>
-        <v>8 × 7</v>
-      </c>
-      <c r="E33" s="6" t="n">
-        <f aca="false">VALUE(MID(A33,7,2))*C33</f>
-        <v>56</v>
-      </c>
-      <c r="F33" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="H33" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="I33" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="J33" s="5"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B34" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="C34" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="D34" s="6" t="str">
-        <f aca="false">"8 × "&amp;C34</f>
-        <v>8 × 7</v>
-      </c>
-      <c r="E34" s="6" t="n">
-        <f aca="false">VALUE(MID(A34,7,2))*C34</f>
-        <v>56</v>
-      </c>
-      <c r="F34" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G34" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="H34" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="I34" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="J34" s="5"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B35" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="C35" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="D35" s="6" t="str">
-        <f aca="false">"8 × "&amp;C35</f>
-        <v>8 × 7</v>
-      </c>
-      <c r="E35" s="6" t="n">
-        <f aca="false">VALUE(MID(A35,7,2))*C35</f>
-        <v>56</v>
-      </c>
-      <c r="F35" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G35" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="H35" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="I35" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="J35" s="5"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J35" s="9"/>
+    </row>
+    <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B36" s="9" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C36" s="9" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D36" s="10" t="str">
         <f aca="false">"8 × "&amp;C36</f>
-        <v>8 × 9</v>
+        <v>8 × 6</v>
       </c>
       <c r="E36" s="10" t="n">
         <f aca="false">VALUE(MID(A36,7,2))*C36</f>
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="F36" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G36" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="H36" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="D37" s="6" t="str">
+        <f aca="false">"8 × "&amp;C37</f>
+        <v>8 × 7</v>
+      </c>
+      <c r="E37" s="6" t="n">
+        <f aca="false">VALUE(MID(A37,7,2))*C37</f>
+        <v>56</v>
+      </c>
+      <c r="F37" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="G36" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="H36" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I36" s="9" t="s">
+      <c r="G37" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H37" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I37" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="J36" s="9"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B37" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="C37" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="D37" s="10" t="str">
-        <f aca="false">"8 × "&amp;C37</f>
-        <v>8 × 9</v>
-      </c>
-      <c r="E37" s="10" t="n">
-        <f aca="false">VALUE(MID(A37,7,2))*C37</f>
-        <v>72</v>
-      </c>
-      <c r="F37" s="9" t="n">
+      <c r="J37" s="5"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="D38" s="6" t="str">
+        <f aca="false">"8 × "&amp;C38</f>
+        <v>8 × 7</v>
+      </c>
+      <c r="E38" s="6" t="n">
+        <f aca="false">VALUE(MID(A38,7,2))*C38</f>
+        <v>56</v>
+      </c>
+      <c r="F38" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G37" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="H37" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I37" s="9" t="s">
+      <c r="G38" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="H38" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I38" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="J37" s="9"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B38" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="C38" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="D38" s="10" t="str">
-        <f aca="false">"8 × "&amp;C38</f>
-        <v>8 × 9</v>
-      </c>
-      <c r="E38" s="10" t="n">
-        <f aca="false">VALUE(MID(A38,7,2))*C38</f>
-        <v>72</v>
-      </c>
-      <c r="F38" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="G38" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="H38" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="I38" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="J38" s="9"/>
+      <c r="J38" s="5"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
         <v>31</v>
       </c>
       <c r="B39" s="5" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C39" s="5" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D39" s="6" t="str">
         <f aca="false">"8 × "&amp;C39</f>
-        <v>8 × 12</v>
+        <v>8 × 7</v>
       </c>
       <c r="E39" s="6" t="n">
         <f aca="false">VALUE(MID(A39,7,2))*C39</f>
-        <v>96</v>
+        <v>56</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="H39" s="8" t="s">
         <v>38</v>
       </c>
       <c r="I39" s="5" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="J39" s="5"/>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
         <v>31</v>
       </c>
       <c r="B40" s="5" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C40" s="5" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D40" s="6" t="str">
         <f aca="false">"8 × "&amp;C40</f>
-        <v>8 × 12</v>
+        <v>8 × 7</v>
       </c>
       <c r="E40" s="6" t="n">
         <f aca="false">VALUE(MID(A40,7,2))*C40</f>
+        <v>56</v>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G40" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="I40" s="5"/>
+      <c r="J40" s="5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B41" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="C41" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="D41" s="10" t="str">
+        <f aca="false">"8 × "&amp;C41</f>
+        <v>8 × 9</v>
+      </c>
+      <c r="E41" s="10" t="n">
+        <f aca="false">VALUE(MID(A41,7,2))*C41</f>
+        <v>72</v>
+      </c>
+      <c r="F41" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="H41" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I41" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="J41" s="9"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B42" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="C42" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="D42" s="10" t="str">
+        <f aca="false">"8 × "&amp;C42</f>
+        <v>8 × 9</v>
+      </c>
+      <c r="E42" s="10" t="n">
+        <f aca="false">VALUE(MID(A42,7,2))*C42</f>
+        <v>72</v>
+      </c>
+      <c r="F42" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G42" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="H42" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I42" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="J42" s="9"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B43" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="C43" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="D43" s="10" t="str">
+        <f aca="false">"8 × "&amp;C43</f>
+        <v>8 × 9</v>
+      </c>
+      <c r="E43" s="10" t="n">
+        <f aca="false">VALUE(MID(A43,7,2))*C43</f>
+        <v>72</v>
+      </c>
+      <c r="F43" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G43" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="F40" s="5" t="n">
+      <c r="H43" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I43" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="J43" s="9"/>
+    </row>
+    <row r="44" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B44" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="C44" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="D44" s="10" t="str">
+        <f aca="false">"8 × "&amp;C44</f>
+        <v>8 × 9</v>
+      </c>
+      <c r="E44" s="10" t="n">
+        <f aca="false">VALUE(MID(A44,7,2))*C44</f>
+        <v>72</v>
+      </c>
+      <c r="F44" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G44" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="H44" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="I44" s="9"/>
+      <c r="J44" s="9" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C45" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D45" s="6" t="str">
+        <f aca="false">"8 × "&amp;C45</f>
+        <v>8 × 12</v>
+      </c>
+      <c r="E45" s="6" t="n">
+        <f aca="false">VALUE(MID(A45,7,2))*C45</f>
+        <v>96</v>
+      </c>
+      <c r="F45" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="H45" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I45" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="J45" s="5"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C46" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D46" s="6" t="str">
+        <f aca="false">"8 × "&amp;C46</f>
+        <v>8 × 12</v>
+      </c>
+      <c r="E46" s="6" t="n">
+        <f aca="false">VALUE(MID(A46,7,2))*C46</f>
+        <v>96</v>
+      </c>
+      <c r="F46" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G40" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="H40" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="I40" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="J40" s="5"/>
-    </row>
-    <row r="41" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B41" s="5" t="n">
+      <c r="G46" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="H46" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I46" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="J46" s="5"/>
+    </row>
+    <row r="47" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B47" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="C41" s="5" t="n">
+      <c r="C47" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="D41" s="6" t="str">
-        <f aca="false">"8 × "&amp;C41</f>
+      <c r="D47" s="6" t="str">
+        <f aca="false">"8 × "&amp;C47</f>
         <v>8 × 12</v>
       </c>
-      <c r="E41" s="6" t="n">
-        <f aca="false">VALUE(MID(A41,7,2))*C41</f>
+      <c r="E47" s="6" t="n">
+        <f aca="false">VALUE(MID(A47,7,2))*C47</f>
         <v>96</v>
       </c>
-      <c r="F41" s="5" t="n">
+      <c r="F47" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G41" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="H41" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="I41" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="J41" s="5"/>
+      <c r="G47" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="H47" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I47" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="J47" s="5"/>
+    </row>
+    <row r="48" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C48" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D48" s="6" t="str">
+        <f aca="false">"8 × "&amp;C48</f>
+        <v>8 × 12</v>
+      </c>
+      <c r="E48" s="6" t="n">
+        <f aca="false">VALUE(MID(A48,7,2))*C48</f>
+        <v>96</v>
+      </c>
+      <c r="F48" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="H48" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="I48" s="5"/>
+      <c r="J48" s="5" t="s">
+        <v>104</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J41"/>
+  <autoFilter ref="A1:J48"/>
   <dataValidations count="3">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H2:H500" type="list">
       <formula1>"oui,non"</formula1>
@@ -2427,10 +2693,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2438,7 +2704,7 @@
         <v>63</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2446,7 +2712,7 @@
         <v>66</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2454,7 +2720,7 @@
         <v>54</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2462,7 +2728,7 @@
         <v>52</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2470,15 +2736,15 @@
         <v>60</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2486,15 +2752,15 @@
         <v>48</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2502,7 +2768,7 @@
         <v>39</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2510,7 +2776,7 @@
         <v>44</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2518,7 +2784,7 @@
         <v>46</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>